<commit_message>
feat: change branding to bloomluxecollection and rename Necklaces to Hamper
</commit_message>
<xml_diff>
--- a/server/database/categories.xlsx
+++ b/server/database/categories.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,12 +407,9 @@
         <v>name</v>
       </c>
       <c r="C1" t="str">
-        <v>description</v>
+        <v>image</v>
       </c>
       <c r="D1" t="str">
-        <v>image</v>
-      </c>
-      <c r="E1" t="str">
         <v>createdAt</v>
       </c>
     </row>
@@ -424,12 +421,9 @@
         <v>Bangles</v>
       </c>
       <c r="C2" t="str">
-        <v>Sleek luxury gold, silver and traditional bridal bangles.</v>
+        <v>https://images.unsplash.com/photo-1611591437281-460bfbe1220a?w=600&amp;auto=format&amp;fit=crop&amp;q=80</v>
       </c>
       <c r="D2" t="str">
-        <v>https://images.unsplash.com/photo-1611591437281-460bfbe1220a?w=600&amp;auto=format&amp;fit=crop&amp;q=80</v>
-      </c>
-      <c r="E2" t="str">
         <v>2026-07-18T11:39:04.043Z</v>
       </c>
     </row>
@@ -441,12 +435,9 @@
         <v>Earrings</v>
       </c>
       <c r="C3" t="str">
-        <v>Timeless diamond solitaires, gold studs, and elegant drops.</v>
+        <v>https://images.unsplash.com/photo-1635767798638-3e25273a8236?w=600&amp;auto=format&amp;fit=crop&amp;q=80</v>
       </c>
       <c r="D3" t="str">
-        <v>https://images.unsplash.com/photo-1635767798638-3e25273a8236?w=600&amp;auto=format&amp;fit=crop&amp;q=80</v>
-      </c>
-      <c r="E3" t="str">
         <v>2026-07-18T11:39:04.043Z</v>
       </c>
     </row>
@@ -458,12 +449,9 @@
         <v>Rings</v>
       </c>
       <c r="C4" t="str">
-        <v>Engagement bands, luxury solitaires, and custom rings.</v>
+        <v>https://images.unsplash.com/photo-1605100804763-247f67b3557e?w=600&amp;auto=format&amp;fit=crop&amp;q=80</v>
       </c>
       <c r="D4" t="str">
-        <v>https://images.unsplash.com/photo-1605100804763-247f67b3557e?w=600&amp;auto=format&amp;fit=crop&amp;q=80</v>
-      </c>
-      <c r="E4" t="str">
         <v>2026-07-18T11:39:04.043Z</v>
       </c>
     </row>
@@ -472,21 +460,18 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>Necklaces</v>
+        <v>Hamper</v>
       </c>
       <c r="C5" t="str">
-        <v>Luxury pendants, gold chokers, and diamond chains.</v>
+        <v>https://images.unsplash.com/photo-1599643478518-a784e5dc4c8f?w=600&amp;auto=format&amp;fit=crop&amp;q=80</v>
       </c>
       <c r="D5" t="str">
-        <v>https://images.unsplash.com/photo-1599643478518-a784e5dc4c8f?w=600&amp;auto=format&amp;fit=crop&amp;q=80</v>
-      </c>
-      <c r="E5" t="str">
         <v>2026-07-18T11:39:04.043Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: synchronize local categories.xlsx Excel database sheet with Atlas
</commit_message>
<xml_diff>
--- a/server/database/categories.xlsx
+++ b/server/database/categories.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -424,7 +424,7 @@
         <v>https://images.unsplash.com/photo-1611591437281-460bfbe1220a?w=600&amp;auto=format&amp;fit=crop&amp;q=80</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-07-18T11:39:04.043Z</v>
+        <v>2026-07-28T04:10:06.474Z</v>
       </c>
     </row>
     <row r="3">
@@ -438,7 +438,7 @@
         <v>https://images.unsplash.com/photo-1635767798638-3e25273a8236?w=600&amp;auto=format&amp;fit=crop&amp;q=80</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-07-18T11:39:04.043Z</v>
+        <v>2026-07-28T04:10:06.475Z</v>
       </c>
     </row>
     <row r="4">
@@ -452,7 +452,7 @@
         <v>https://images.unsplash.com/photo-1605100804763-247f67b3557e?w=600&amp;auto=format&amp;fit=crop&amp;q=80</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-07-18T11:39:04.043Z</v>
+        <v>2026-07-28T04:10:06.475Z</v>
       </c>
     </row>
     <row r="5">
@@ -466,12 +466,26 @@
         <v>https://images.unsplash.com/photo-1599643478518-a784e5dc4c8f?w=600&amp;auto=format&amp;fit=crop&amp;q=80</v>
       </c>
       <c r="D5" t="str">
-        <v>2026-07-18T11:39:04.043Z</v>
+        <v>2026-07-28T04:10:06.475Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Watches</v>
+      </c>
+      <c r="C6" t="str">
+        <v>https://images.unsplash.com/photo-1523275335684-37898b6baf30?w=600&amp;auto=format&amp;fit=crop&amp;q=80</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2026-07-28T04:10:06.475Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>